<commit_message>
260818 after code review before coding
</commit_message>
<xml_diff>
--- a/order book.xlsx
+++ b/order book.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7398" uniqueCount="3179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7418" uniqueCount="3194">
   <si>
     <t>* 부가세(VAT) 포함 금액 기재 / 서브원 외에는 물품 "사진" 필수</t>
   </si>
@@ -9613,6 +9613,64 @@
   </si>
   <si>
     <t>o</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>o</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>o</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>O</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>o</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>abcam</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>20 uL</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ab92536</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lot No.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ThermoFisher</t>
+  </si>
+  <si>
+    <t>M30550</t>
+  </si>
+  <si>
+    <t>o</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>8/13</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>dd</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>sdfg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>46eoier</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -9933,7 +9991,7 @@
       <charset val="129"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9991,12 +10049,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6F7E6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -10481,7 +10533,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -11125,9 +11177,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -11521,174 +11570,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21.75" customHeight="1">
-      <c r="A1" s="221" t="s">
+      <c r="A1" s="220" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="222"/>
-      <c r="C1" s="223"/>
-      <c r="D1" s="223"/>
-      <c r="E1" s="223"/>
-      <c r="F1" s="223"/>
-      <c r="G1" s="223"/>
-      <c r="H1" s="223"/>
-      <c r="I1" s="223"/>
-      <c r="J1" s="224"/>
-      <c r="K1" s="222"/>
-      <c r="L1" s="222"/>
-      <c r="M1" s="223"/>
+      <c r="B1" s="221"/>
+      <c r="C1" s="222"/>
+      <c r="D1" s="222"/>
+      <c r="E1" s="222"/>
+      <c r="F1" s="222"/>
+      <c r="G1" s="222"/>
+      <c r="H1" s="222"/>
+      <c r="I1" s="222"/>
+      <c r="J1" s="223"/>
+      <c r="K1" s="221"/>
+      <c r="L1" s="221"/>
+      <c r="M1" s="222"/>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="238" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="240"/>
-      <c r="C2" s="240"/>
-      <c r="D2" s="240"/>
-      <c r="E2" s="240"/>
-      <c r="F2" s="240"/>
-      <c r="G2" s="240"/>
-      <c r="H2" s="240"/>
-      <c r="I2" s="240"/>
-      <c r="J2" s="240"/>
-      <c r="K2" s="240"/>
-      <c r="L2" s="240"/>
-      <c r="M2" s="241"/>
+      <c r="B2" s="239"/>
+      <c r="C2" s="239"/>
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="239"/>
+      <c r="H2" s="239"/>
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
+      <c r="M2" s="240"/>
     </row>
     <row r="3" spans="1:19" ht="19.5" customHeight="1">
-      <c r="A3" s="236" t="s">
+      <c r="A3" s="235" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="237"/>
-      <c r="C3" s="237"/>
-      <c r="D3" s="237"/>
-      <c r="E3" s="237"/>
-      <c r="F3" s="237"/>
-      <c r="G3" s="237"/>
-      <c r="H3" s="237"/>
-      <c r="I3" s="237"/>
-      <c r="J3" s="237"/>
-      <c r="K3" s="237"/>
-      <c r="L3" s="237"/>
-      <c r="M3" s="237"/>
+      <c r="B3" s="236"/>
+      <c r="C3" s="236"/>
+      <c r="D3" s="236"/>
+      <c r="E3" s="236"/>
+      <c r="F3" s="236"/>
+      <c r="G3" s="236"/>
+      <c r="H3" s="236"/>
+      <c r="I3" s="236"/>
+      <c r="J3" s="236"/>
+      <c r="K3" s="236"/>
+      <c r="L3" s="236"/>
+      <c r="M3" s="236"/>
     </row>
     <row r="4" spans="1:19" s="5" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A4" s="233" t="s">
+      <c r="A4" s="232" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="234"/>
-      <c r="C4" s="234"/>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
-      <c r="M4" s="235"/>
+      <c r="B4" s="233"/>
+      <c r="C4" s="233"/>
+      <c r="D4" s="233"/>
+      <c r="E4" s="233"/>
+      <c r="F4" s="233"/>
+      <c r="G4" s="233"/>
+      <c r="H4" s="233"/>
+      <c r="I4" s="233"/>
+      <c r="J4" s="233"/>
+      <c r="K4" s="233"/>
+      <c r="L4" s="233"/>
+      <c r="M4" s="234"/>
     </row>
     <row r="5" spans="1:19" s="5" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A5" s="225" t="s">
+      <c r="A5" s="224" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="226"/>
-      <c r="C5" s="226"/>
-      <c r="D5" s="226"/>
-      <c r="E5" s="226"/>
-      <c r="F5" s="226"/>
-      <c r="G5" s="226"/>
-      <c r="H5" s="226"/>
-      <c r="I5" s="226"/>
-      <c r="J5" s="226"/>
-      <c r="K5" s="226"/>
-      <c r="L5" s="226"/>
-      <c r="M5" s="227"/>
+      <c r="B5" s="225"/>
+      <c r="C5" s="225"/>
+      <c r="D5" s="225"/>
+      <c r="E5" s="225"/>
+      <c r="F5" s="225"/>
+      <c r="G5" s="225"/>
+      <c r="H5" s="225"/>
+      <c r="I5" s="225"/>
+      <c r="J5" s="225"/>
+      <c r="K5" s="225"/>
+      <c r="L5" s="225"/>
+      <c r="M5" s="226"/>
     </row>
     <row r="6" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A6" s="229" t="s">
+      <c r="A6" s="228" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="230"/>
-      <c r="C6" s="230"/>
-      <c r="D6" s="230"/>
-      <c r="E6" s="230"/>
-      <c r="F6" s="230"/>
-      <c r="G6" s="230"/>
-      <c r="H6" s="230"/>
-      <c r="I6" s="230"/>
-      <c r="J6" s="230"/>
-      <c r="K6" s="230"/>
-      <c r="L6" s="230"/>
-      <c r="M6" s="231"/>
+      <c r="B6" s="229"/>
+      <c r="C6" s="229"/>
+      <c r="D6" s="229"/>
+      <c r="E6" s="229"/>
+      <c r="F6" s="229"/>
+      <c r="G6" s="229"/>
+      <c r="H6" s="229"/>
+      <c r="I6" s="229"/>
+      <c r="J6" s="229"/>
+      <c r="K6" s="229"/>
+      <c r="L6" s="229"/>
+      <c r="M6" s="230"/>
     </row>
     <row r="7" spans="1:19" s="5" customFormat="1" ht="25.5" hidden="1" customHeight="1">
-      <c r="A7" s="238" t="s">
+      <c r="A7" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="219"/>
-      <c r="C7" s="219"/>
-      <c r="D7" s="219"/>
-      <c r="E7" s="219"/>
-      <c r="F7" s="219"/>
-      <c r="G7" s="219"/>
-      <c r="H7" s="219"/>
-      <c r="I7" s="219"/>
-      <c r="J7" s="219"/>
-      <c r="K7" s="219"/>
-      <c r="L7" s="219"/>
-      <c r="M7" s="219"/>
+      <c r="B7" s="218"/>
+      <c r="C7" s="218"/>
+      <c r="D7" s="218"/>
+      <c r="E7" s="218"/>
+      <c r="F7" s="218"/>
+      <c r="G7" s="218"/>
+      <c r="H7" s="218"/>
+      <c r="I7" s="218"/>
+      <c r="J7" s="218"/>
+      <c r="K7" s="218"/>
+      <c r="L7" s="218"/>
+      <c r="M7" s="218"/>
     </row>
     <row r="8" spans="1:19" s="5" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A8" s="228" t="s">
+      <c r="A8" s="227" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="219"/>
-      <c r="C8" s="219"/>
-      <c r="D8" s="219"/>
-      <c r="E8" s="219"/>
-      <c r="F8" s="219"/>
-      <c r="G8" s="219"/>
-      <c r="H8" s="219"/>
-      <c r="I8" s="219"/>
-      <c r="J8" s="219"/>
-      <c r="K8" s="219"/>
-      <c r="L8" s="219"/>
-      <c r="M8" s="219"/>
+      <c r="B8" s="218"/>
+      <c r="C8" s="218"/>
+      <c r="D8" s="218"/>
+      <c r="E8" s="218"/>
+      <c r="F8" s="218"/>
+      <c r="G8" s="218"/>
+      <c r="H8" s="218"/>
+      <c r="I8" s="218"/>
+      <c r="J8" s="218"/>
+      <c r="K8" s="218"/>
+      <c r="L8" s="218"/>
+      <c r="M8" s="218"/>
     </row>
     <row r="9" spans="1:19" s="5" customFormat="1" ht="28.5" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A9" s="232" t="s">
+      <c r="A9" s="231" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="219"/>
-      <c r="C9" s="219"/>
-      <c r="D9" s="219"/>
-      <c r="E9" s="219"/>
-      <c r="F9" s="219"/>
-      <c r="G9" s="219"/>
-      <c r="H9" s="219"/>
-      <c r="I9" s="219"/>
-      <c r="J9" s="219"/>
-      <c r="K9" s="219"/>
-      <c r="L9" s="219"/>
-      <c r="M9" s="219"/>
+      <c r="B9" s="218"/>
+      <c r="C9" s="218"/>
+      <c r="D9" s="218"/>
+      <c r="E9" s="218"/>
+      <c r="F9" s="218"/>
+      <c r="G9" s="218"/>
+      <c r="H9" s="218"/>
+      <c r="I9" s="218"/>
+      <c r="J9" s="218"/>
+      <c r="K9" s="218"/>
+      <c r="L9" s="218"/>
+      <c r="M9" s="218"/>
     </row>
     <row r="10" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A10" s="218" t="s">
+      <c r="A10" s="217" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="219"/>
-      <c r="C10" s="219"/>
-      <c r="D10" s="219"/>
-      <c r="E10" s="219"/>
-      <c r="F10" s="219"/>
-      <c r="G10" s="219"/>
-      <c r="H10" s="219"/>
-      <c r="I10" s="219"/>
-      <c r="J10" s="219"/>
-      <c r="K10" s="219"/>
-      <c r="L10" s="219"/>
-      <c r="M10" s="220"/>
+      <c r="B10" s="218"/>
+      <c r="C10" s="218"/>
+      <c r="D10" s="218"/>
+      <c r="E10" s="218"/>
+      <c r="F10" s="218"/>
+      <c r="G10" s="218"/>
+      <c r="H10" s="218"/>
+      <c r="I10" s="218"/>
+      <c r="J10" s="218"/>
+      <c r="K10" s="218"/>
+      <c r="L10" s="218"/>
+      <c r="M10" s="219"/>
     </row>
     <row r="11" spans="1:19" s="5" customFormat="1" ht="17.25" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -37350,109 +37399,109 @@
     <col min="21" max="16384" width="7.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="5" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A1" s="233" t="s">
+    <row r="1" spans="1:20" s="5" customFormat="1" ht="26.25" customHeight="1">
+      <c r="A1" s="232" t="s">
         <v>2145</v>
       </c>
-      <c r="B1" s="234"/>
-      <c r="C1" s="234"/>
-      <c r="D1" s="234"/>
-      <c r="E1" s="234"/>
-      <c r="F1" s="234"/>
-      <c r="G1" s="234"/>
-      <c r="H1" s="234"/>
-      <c r="I1" s="234"/>
-      <c r="J1" s="234"/>
-      <c r="K1" s="234"/>
-      <c r="L1" s="234"/>
-      <c r="M1" s="235"/>
-    </row>
-    <row r="2" spans="1:19" s="5" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A2" s="225" t="s">
+      <c r="B1" s="233"/>
+      <c r="C1" s="233"/>
+      <c r="D1" s="233"/>
+      <c r="E1" s="233"/>
+      <c r="F1" s="233"/>
+      <c r="G1" s="233"/>
+      <c r="H1" s="233"/>
+      <c r="I1" s="233"/>
+      <c r="J1" s="233"/>
+      <c r="K1" s="233"/>
+      <c r="L1" s="233"/>
+      <c r="M1" s="234"/>
+    </row>
+    <row r="2" spans="1:20" s="5" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A2" s="224" t="s">
         <v>2146</v>
       </c>
-      <c r="B2" s="226"/>
-      <c r="C2" s="226"/>
-      <c r="D2" s="226"/>
-      <c r="E2" s="226"/>
-      <c r="F2" s="226"/>
-      <c r="G2" s="226"/>
-      <c r="H2" s="226"/>
-      <c r="I2" s="226"/>
-      <c r="J2" s="226"/>
-      <c r="K2" s="226"/>
-      <c r="L2" s="226"/>
-      <c r="M2" s="227"/>
-    </row>
-    <row r="3" spans="1:19" s="5" customFormat="1" ht="27" hidden="1" customHeight="1">
-      <c r="A3" s="238" t="s">
+      <c r="B2" s="225"/>
+      <c r="C2" s="225"/>
+      <c r="D2" s="225"/>
+      <c r="E2" s="225"/>
+      <c r="F2" s="225"/>
+      <c r="G2" s="225"/>
+      <c r="H2" s="225"/>
+      <c r="I2" s="225"/>
+      <c r="J2" s="225"/>
+      <c r="K2" s="225"/>
+      <c r="L2" s="225"/>
+      <c r="M2" s="226"/>
+    </row>
+    <row r="3" spans="1:20" s="5" customFormat="1" ht="27" hidden="1" customHeight="1">
+      <c r="A3" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="219"/>
-      <c r="C3" s="219"/>
-      <c r="D3" s="219"/>
-      <c r="E3" s="219"/>
-      <c r="F3" s="219"/>
-      <c r="G3" s="219"/>
-      <c r="H3" s="219"/>
-      <c r="I3" s="219"/>
-      <c r="J3" s="219"/>
-      <c r="K3" s="219"/>
-      <c r="L3" s="219"/>
-      <c r="M3" s="219"/>
-    </row>
-    <row r="4" spans="1:19" s="5" customFormat="1" ht="41.25" hidden="1" customHeight="1">
-      <c r="A4" s="228" t="s">
+      <c r="B3" s="218"/>
+      <c r="C3" s="218"/>
+      <c r="D3" s="218"/>
+      <c r="E3" s="218"/>
+      <c r="F3" s="218"/>
+      <c r="G3" s="218"/>
+      <c r="H3" s="218"/>
+      <c r="I3" s="218"/>
+      <c r="J3" s="218"/>
+      <c r="K3" s="218"/>
+      <c r="L3" s="218"/>
+      <c r="M3" s="218"/>
+    </row>
+    <row r="4" spans="1:20" s="5" customFormat="1" ht="41.25" hidden="1" customHeight="1">
+      <c r="A4" s="227" t="s">
         <v>2147</v>
       </c>
-      <c r="B4" s="219"/>
-      <c r="C4" s="219"/>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
-      <c r="M4" s="219"/>
-    </row>
-    <row r="5" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1">
-      <c r="A5" s="232" t="s">
+      <c r="B4" s="218"/>
+      <c r="C4" s="218"/>
+      <c r="D4" s="218"/>
+      <c r="E4" s="218"/>
+      <c r="F4" s="218"/>
+      <c r="G4" s="218"/>
+      <c r="H4" s="218"/>
+      <c r="I4" s="218"/>
+      <c r="J4" s="218"/>
+      <c r="K4" s="218"/>
+      <c r="L4" s="218"/>
+      <c r="M4" s="218"/>
+    </row>
+    <row r="5" spans="1:20" s="5" customFormat="1" ht="21.75" customHeight="1">
+      <c r="A5" s="231" t="s">
         <v>2148</v>
       </c>
-      <c r="B5" s="219"/>
-      <c r="C5" s="219"/>
-      <c r="D5" s="219"/>
-      <c r="E5" s="219"/>
-      <c r="F5" s="219"/>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
-      <c r="J5" s="219"/>
-      <c r="K5" s="219"/>
-      <c r="L5" s="219"/>
-      <c r="M5" s="219"/>
-    </row>
-    <row r="6" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1">
-      <c r="A6" s="218" t="s">
+      <c r="B5" s="218"/>
+      <c r="C5" s="218"/>
+      <c r="D5" s="218"/>
+      <c r="E5" s="218"/>
+      <c r="F5" s="218"/>
+      <c r="G5" s="218"/>
+      <c r="H5" s="218"/>
+      <c r="I5" s="218"/>
+      <c r="J5" s="218"/>
+      <c r="K5" s="218"/>
+      <c r="L5" s="218"/>
+      <c r="M5" s="218"/>
+    </row>
+    <row r="6" spans="1:20" s="5" customFormat="1" ht="21.75" customHeight="1">
+      <c r="A6" s="217" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="219"/>
-      <c r="C6" s="219"/>
-      <c r="D6" s="219"/>
-      <c r="E6" s="219"/>
-      <c r="F6" s="219"/>
-      <c r="G6" s="219"/>
-      <c r="H6" s="219"/>
-      <c r="I6" s="219"/>
-      <c r="J6" s="219"/>
-      <c r="K6" s="219"/>
-      <c r="L6" s="219"/>
-      <c r="M6" s="220"/>
-    </row>
-    <row r="7" spans="1:19" s="5" customFormat="1" ht="17.25" customHeight="1">
+      <c r="B6" s="218"/>
+      <c r="C6" s="218"/>
+      <c r="D6" s="218"/>
+      <c r="E6" s="218"/>
+      <c r="F6" s="218"/>
+      <c r="G6" s="218"/>
+      <c r="H6" s="218"/>
+      <c r="I6" s="218"/>
+      <c r="J6" s="218"/>
+      <c r="K6" s="218"/>
+      <c r="L6" s="218"/>
+      <c r="M6" s="219"/>
+    </row>
+    <row r="7" spans="1:20" s="5" customFormat="1" ht="17.25" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -37510,8 +37559,11 @@
       <c r="S7" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+      <c r="T7" s="5" t="s">
+        <v>3186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A8" s="168" t="s">
         <v>2150</v>
       </c>
@@ -37538,7 +37590,7 @@
       <c r="L8" s="173"/>
       <c r="M8" s="174"/>
     </row>
-    <row r="9" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="9" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A9" s="168" t="s">
         <v>2153</v>
       </c>
@@ -37565,7 +37617,7 @@
       <c r="L9" s="173"/>
       <c r="M9" s="174"/>
     </row>
-    <row r="10" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="10" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A10" s="168" t="s">
         <v>2155</v>
       </c>
@@ -37592,7 +37644,7 @@
       <c r="L10" s="173"/>
       <c r="M10" s="174"/>
     </row>
-    <row r="11" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="11" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A11" s="168" t="s">
         <v>2158</v>
       </c>
@@ -37617,7 +37669,7 @@
       <c r="L11" s="173"/>
       <c r="M11" s="174"/>
     </row>
-    <row r="12" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="12" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A12" s="168" t="s">
         <v>2159</v>
       </c>
@@ -37644,7 +37696,7 @@
       <c r="L12" s="173"/>
       <c r="M12" s="174"/>
     </row>
-    <row r="13" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="13" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A13" s="168" t="s">
         <v>2161</v>
       </c>
@@ -37671,7 +37723,7 @@
       <c r="L13" s="173"/>
       <c r="M13" s="174"/>
     </row>
-    <row r="14" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="14" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A14" s="168" t="s">
         <v>2163</v>
       </c>
@@ -37697,7 +37749,7 @@
       <c r="L14" s="173"/>
       <c r="M14" s="174"/>
     </row>
-    <row r="15" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="15" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A15" s="168" t="s">
         <v>2165</v>
       </c>
@@ -37724,7 +37776,7 @@
       <c r="L15" s="173"/>
       <c r="M15" s="174"/>
     </row>
-    <row r="16" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="16" spans="1:20" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A16" s="168" t="s">
         <v>2166</v>
       </c>
@@ -37755,7 +37807,7 @@
       <c r="N16" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O16" s="217" t="s">
+      <c r="O16" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
@@ -37898,7 +37950,7 @@
       <c r="N21" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O21" s="217" t="s">
+      <c r="O21" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P21" s="175" t="s">
@@ -37945,7 +37997,7 @@
       <c r="N22" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O22" s="217" t="s">
+      <c r="O22" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P22" s="175" t="s">
@@ -38226,7 +38278,7 @@
       <c r="N32" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O32" s="217" t="s">
+      <c r="O32" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P32" s="175" t="s">
@@ -38460,7 +38512,7 @@
       <c r="N40" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O40" s="217" t="s">
+      <c r="O40" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
@@ -38601,7 +38653,7 @@
       <c r="N45" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O45" s="217" t="s">
+      <c r="O45" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P45" s="175" t="s">
@@ -38673,7 +38725,7 @@
       <c r="N47" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O47" s="217" t="s">
+      <c r="O47" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P47" s="175" t="s">
@@ -38774,7 +38826,7 @@
       <c r="N50" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O50" s="217" t="s">
+      <c r="O50" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
@@ -38838,7 +38890,7 @@
       <c r="N52" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O52" s="217" t="s">
+      <c r="O52" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
@@ -38950,7 +39002,7 @@
       <c r="N56" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O56" s="217" t="s">
+      <c r="O56" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
@@ -39007,6 +39059,12 @@
       <c r="K58" s="172"/>
       <c r="L58" s="172"/>
       <c r="M58" s="174"/>
+      <c r="N58" s="175" t="s">
+        <v>3180</v>
+      </c>
+      <c r="O58" s="175" t="s">
+        <v>3180</v>
+      </c>
     </row>
     <row r="59" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A59" s="168" t="s">
@@ -39059,6 +39117,12 @@
       <c r="K60" s="172"/>
       <c r="L60" s="172"/>
       <c r="M60" s="174"/>
+      <c r="N60" s="175" t="s">
+        <v>3181</v>
+      </c>
+      <c r="O60" s="175" t="s">
+        <v>3181</v>
+      </c>
     </row>
     <row r="61" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A61" s="168" t="s">
@@ -39172,7 +39236,7 @@
       <c r="N64" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O64" s="217" t="s">
+      <c r="O64" s="175" t="s">
         <v>2015</v>
       </c>
       <c r="P64" s="175">
@@ -39188,7 +39252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="65" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A65" s="168" t="s">
         <v>2261</v>
       </c>
@@ -39215,7 +39279,7 @@
       <c r="L65" s="169"/>
       <c r="M65" s="168"/>
     </row>
-    <row r="66" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="66" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A66" s="168" t="s">
         <v>2263</v>
       </c>
@@ -39241,8 +39305,26 @@
       <c r="K66" s="169"/>
       <c r="L66" s="169"/>
       <c r="M66" s="168"/>
-    </row>
-    <row r="67" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+      <c r="N66" s="175" t="s">
+        <v>3182</v>
+      </c>
+      <c r="O66" s="175" t="s">
+        <v>3182</v>
+      </c>
+      <c r="P66" s="175" t="s">
+        <v>3183</v>
+      </c>
+      <c r="Q66" s="175">
+        <v>1</v>
+      </c>
+      <c r="R66" s="175" t="s">
+        <v>3184</v>
+      </c>
+      <c r="S66" s="175" t="s">
+        <v>3185</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A67" s="168" t="s">
         <v>2265</v>
       </c>
@@ -39273,11 +39355,11 @@
       <c r="N67" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O67" s="217" t="s">
+      <c r="O67" s="175" t="s">
         <v>2015</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="68" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A68" s="168" t="s">
         <v>2267</v>
       </c>
@@ -39304,7 +39386,7 @@
       <c r="L68" s="169"/>
       <c r="M68" s="168"/>
     </row>
-    <row r="69" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="69" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A69" s="168" t="s">
         <v>2269</v>
       </c>
@@ -39331,7 +39413,7 @@
       <c r="L69" s="169"/>
       <c r="M69" s="168"/>
     </row>
-    <row r="70" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="70" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A70" s="168" t="s">
         <v>2271</v>
       </c>
@@ -39357,8 +39439,14 @@
       <c r="K70" s="169"/>
       <c r="L70" s="169"/>
       <c r="M70" s="168"/>
-    </row>
-    <row r="71" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+      <c r="N70" s="175" t="s">
+        <v>3179</v>
+      </c>
+      <c r="O70" s="175" t="s">
+        <v>3179</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A71" s="168" t="s">
         <v>2275</v>
       </c>
@@ -39385,7 +39473,7 @@
       <c r="L71" s="169"/>
       <c r="M71" s="168"/>
     </row>
-    <row r="72" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="72" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A72" s="168" t="s">
         <v>2277</v>
       </c>
@@ -39412,7 +39500,7 @@
       <c r="L72" s="169"/>
       <c r="M72" s="168"/>
     </row>
-    <row r="73" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="73" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A73" s="168" t="s">
         <v>2279</v>
       </c>
@@ -39439,7 +39527,7 @@
       <c r="L73" s="169"/>
       <c r="M73" s="168"/>
     </row>
-    <row r="74" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="74" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A74" s="168" t="s">
         <v>2282</v>
       </c>
@@ -39466,7 +39554,7 @@
       <c r="L74" s="169"/>
       <c r="M74" s="168"/>
     </row>
-    <row r="75" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="75" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A75" s="168" t="s">
         <v>2284</v>
       </c>
@@ -39493,7 +39581,7 @@
       <c r="L75" s="169"/>
       <c r="M75" s="168"/>
     </row>
-    <row r="76" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="76" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A76" s="168" t="s">
         <v>2287</v>
       </c>
@@ -39520,7 +39608,7 @@
       <c r="L76" s="169"/>
       <c r="M76" s="168"/>
     </row>
-    <row r="77" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="77" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A77" s="168" t="s">
         <v>2288</v>
       </c>
@@ -39547,7 +39635,7 @@
       <c r="L77" s="169"/>
       <c r="M77" s="168"/>
     </row>
-    <row r="78" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="78" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A78" s="168" t="s">
         <v>2290</v>
       </c>
@@ -39574,7 +39662,7 @@
       <c r="L78" s="169"/>
       <c r="M78" s="168"/>
     </row>
-    <row r="79" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="79" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A79" s="168" t="s">
         <v>2292</v>
       </c>
@@ -39601,7 +39689,7 @@
       <c r="L79" s="169"/>
       <c r="M79" s="168"/>
     </row>
-    <row r="80" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="80" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A80" s="168" t="s">
         <v>2294</v>
       </c>
@@ -39767,7 +39855,7 @@
       <c r="N85" s="175" t="s">
         <v>2015</v>
       </c>
-      <c r="O85" s="217" t="s">
+      <c r="O85" s="175" t="s">
         <v>3152</v>
       </c>
       <c r="Q85" s="175">
@@ -40429,7 +40517,7 @@
       <c r="N109" s="175" t="s">
         <v>3148</v>
       </c>
-      <c r="O109" s="217" t="s">
+      <c r="O109" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -40759,7 +40847,7 @@
       <c r="N121" s="175" t="s">
         <v>3139</v>
       </c>
-      <c r="O121" s="217" t="s">
+      <c r="O121" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -41066,7 +41154,7 @@
       <c r="N132" s="175" t="s">
         <v>3150</v>
       </c>
-      <c r="O132" s="217" t="s">
+      <c r="O132" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -41352,7 +41440,7 @@
       <c r="N142" s="175" t="s">
         <v>3139</v>
       </c>
-      <c r="O142" s="217" t="s">
+      <c r="O142" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -41441,7 +41529,7 @@
       <c r="N145" s="175" t="s">
         <v>3139</v>
       </c>
-      <c r="O145" s="217" t="s">
+      <c r="O145" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -46323,7 +46411,7 @@
       <c r="N322" s="175" t="s">
         <v>3169</v>
       </c>
-      <c r="O322" s="217" t="s">
+      <c r="O322" s="175" t="s">
         <v>3169</v>
       </c>
       <c r="P322" s="175" t="s">
@@ -46428,7 +46516,7 @@
       <c r="N325" s="175" t="s">
         <v>3165</v>
       </c>
-      <c r="O325" s="217" t="s">
+      <c r="O325" s="175" t="s">
         <v>3165</v>
       </c>
       <c r="P325" s="175" t="s">
@@ -47039,7 +47127,7 @@
       <c r="N346" s="175" t="s">
         <v>3160</v>
       </c>
-      <c r="O346" s="217" t="s">
+      <c r="O346" s="175" t="s">
         <v>3160</v>
       </c>
       <c r="P346" s="175" t="s">
@@ -47086,7 +47174,7 @@
       <c r="N347" s="175" t="s">
         <v>3157</v>
       </c>
-      <c r="O347" s="217" t="s">
+      <c r="O347" s="175" t="s">
         <v>3157</v>
       </c>
       <c r="P347" s="175" t="s">
@@ -47295,7 +47383,7 @@
       <c r="N354" s="175" t="s">
         <v>3162</v>
       </c>
-      <c r="O354" s="217" t="s">
+      <c r="O354" s="175" t="s">
         <v>3162</v>
       </c>
       <c r="P354" s="175" t="s">
@@ -49862,7 +49950,7 @@
       <c r="N447" s="175" t="s">
         <v>3178</v>
       </c>
-      <c r="O447" s="217" t="s">
+      <c r="O447" s="175" t="s">
         <v>3178</v>
       </c>
     </row>
@@ -50291,7 +50379,7 @@
       <c r="N462" s="175" t="s">
         <v>3153</v>
       </c>
-      <c r="O462" s="217" t="s">
+      <c r="O462" s="175" t="s">
         <v>3153</v>
       </c>
     </row>
@@ -50324,7 +50412,7 @@
       <c r="N463" s="175" t="s">
         <v>3177</v>
       </c>
-      <c r="O463" s="217" t="s">
+      <c r="O463" s="175" t="s">
         <v>3177</v>
       </c>
     </row>
@@ -50523,7 +50611,7 @@
       <c r="N470" s="175" t="s">
         <v>3173</v>
       </c>
-      <c r="O470" s="217" t="s">
+      <c r="O470" s="175" t="s">
         <v>3173</v>
       </c>
       <c r="P470" s="175" t="s">
@@ -50595,7 +50683,7 @@
       <c r="N472" s="175" t="s">
         <v>3154</v>
       </c>
-      <c r="O472" s="217" t="s">
+      <c r="O472" s="175" t="s">
         <v>3154</v>
       </c>
     </row>
@@ -50707,7 +50795,7 @@
       <c r="N476" s="175" t="s">
         <v>3156</v>
       </c>
-      <c r="O476" s="217" t="s">
+      <c r="O476" s="175" t="s">
         <v>3156</v>
       </c>
     </row>
@@ -50769,7 +50857,7 @@
       <c r="N478" s="175" t="s">
         <v>3139</v>
       </c>
-      <c r="O478" s="217" t="s">
+      <c r="O478" s="175" t="s">
         <v>3139</v>
       </c>
     </row>
@@ -50829,11 +50917,11 @@
       <c r="N480" s="175" t="s">
         <v>3155</v>
       </c>
-      <c r="O480" s="217" t="s">
+      <c r="O480" s="175" t="s">
         <v>3155</v>
       </c>
     </row>
-    <row r="481" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="481" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A481" s="168" t="s">
         <v>3070</v>
       </c>
@@ -50860,7 +50948,7 @@
       <c r="L481" s="169"/>
       <c r="M481" s="168"/>
     </row>
-    <row r="482" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="482" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A482" s="168" t="s">
         <v>3071</v>
       </c>
@@ -50887,7 +50975,7 @@
       <c r="L482" s="169"/>
       <c r="M482" s="168"/>
     </row>
-    <row r="483" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="483" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A483" s="168" t="s">
         <v>3073</v>
       </c>
@@ -50912,7 +51000,7 @@
       <c r="L483" s="169"/>
       <c r="M483" s="168"/>
     </row>
-    <row r="484" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="484" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A484" s="168" t="s">
         <v>3075</v>
       </c>
@@ -50941,7 +51029,7 @@
       <c r="L484" s="169"/>
       <c r="M484" s="168"/>
     </row>
-    <row r="485" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="485" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A485" s="168" t="s">
         <v>3077</v>
       </c>
@@ -50966,7 +51054,7 @@
       <c r="L485" s="169"/>
       <c r="M485" s="168"/>
     </row>
-    <row r="486" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="486" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A486" s="168" t="s">
         <v>3079</v>
       </c>
@@ -50993,24 +51081,51 @@
       <c r="L486" s="169"/>
       <c r="M486" s="168"/>
     </row>
-    <row r="487" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="487" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A487" s="168" t="s">
         <v>3082</v>
       </c>
-      <c r="B487" s="169"/>
-      <c r="C487" s="168"/>
-      <c r="D487" s="168"/>
+      <c r="B487" s="169" t="s">
+        <v>3190</v>
+      </c>
+      <c r="C487" s="168" t="s">
+        <v>3191</v>
+      </c>
+      <c r="D487" s="168" t="s">
+        <v>3192</v>
+      </c>
       <c r="E487" s="168"/>
-      <c r="F487" s="168"/>
-      <c r="G487" s="168"/>
-      <c r="H487" s="168"/>
+      <c r="F487" s="175" t="s">
+        <v>3193</v>
+      </c>
       <c r="I487" s="168"/>
       <c r="J487" s="192"/>
       <c r="K487" s="169"/>
       <c r="L487" s="169"/>
       <c r="M487" s="168"/>
-    </row>
-    <row r="488" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+      <c r="N487" s="175" t="s">
+        <v>3189</v>
+      </c>
+      <c r="O487" s="175" t="s">
+        <v>3139</v>
+      </c>
+      <c r="P487" s="168" t="s">
+        <v>3187</v>
+      </c>
+      <c r="Q487" s="175">
+        <v>1</v>
+      </c>
+      <c r="R487" s="175">
+        <v>11</v>
+      </c>
+      <c r="S487" s="168" t="s">
+        <v>3188</v>
+      </c>
+      <c r="T487" s="168">
+        <v>2291655</v>
+      </c>
+    </row>
+    <row r="488" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A488" s="168" t="s">
         <v>3083</v>
       </c>
@@ -51027,7 +51142,7 @@
       <c r="L488" s="169"/>
       <c r="M488" s="168"/>
     </row>
-    <row r="489" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="489" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A489" s="168" t="s">
         <v>3084</v>
       </c>
@@ -51044,7 +51159,7 @@
       <c r="L489" s="169"/>
       <c r="M489" s="168"/>
     </row>
-    <row r="490" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="490" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A490" s="168" t="s">
         <v>3085</v>
       </c>
@@ -51061,7 +51176,7 @@
       <c r="L490" s="169"/>
       <c r="M490" s="168"/>
     </row>
-    <row r="491" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="491" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A491" s="168" t="s">
         <v>3086</v>
       </c>
@@ -51078,7 +51193,7 @@
       <c r="L491" s="169"/>
       <c r="M491" s="168"/>
     </row>
-    <row r="492" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="492" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A492" s="168" t="s">
         <v>3087</v>
       </c>
@@ -51095,7 +51210,7 @@
       <c r="L492" s="169"/>
       <c r="M492" s="168"/>
     </row>
-    <row r="493" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="493" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A493" s="168" t="s">
         <v>3088</v>
       </c>
@@ -51112,7 +51227,7 @@
       <c r="L493" s="169"/>
       <c r="M493" s="168"/>
     </row>
-    <row r="494" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="494" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A494" s="168" t="s">
         <v>3089</v>
       </c>
@@ -51129,7 +51244,7 @@
       <c r="L494" s="169"/>
       <c r="M494" s="168"/>
     </row>
-    <row r="495" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="495" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A495" s="168" t="s">
         <v>3090</v>
       </c>
@@ -51146,7 +51261,7 @@
       <c r="L495" s="169"/>
       <c r="M495" s="168"/>
     </row>
-    <row r="496" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="496" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A496" s="168" t="s">
         <v>3091</v>
       </c>
@@ -51707,7 +51822,7 @@
       <c r="L528" s="169"/>
       <c r="M528" s="168"/>
     </row>
-    <row r="529" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="529" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A529" s="168" t="s">
         <v>3124</v>
       </c>
@@ -51724,7 +51839,7 @@
       <c r="L529" s="169"/>
       <c r="M529" s="168"/>
     </row>
-    <row r="530" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="530" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A530" s="168" t="s">
         <v>3125</v>
       </c>
@@ -51741,7 +51856,7 @@
       <c r="L530" s="169"/>
       <c r="M530" s="168"/>
     </row>
-    <row r="531" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="531" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A531" s="168" t="s">
         <v>3126</v>
       </c>
@@ -51758,7 +51873,7 @@
       <c r="L531" s="169"/>
       <c r="M531" s="168"/>
     </row>
-    <row r="532" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="532" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A532" s="168" t="s">
         <v>3127</v>
       </c>
@@ -51775,7 +51890,7 @@
       <c r="L532" s="169"/>
       <c r="M532" s="168"/>
     </row>
-    <row r="533" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="533" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A533" s="168" t="s">
         <v>3128</v>
       </c>
@@ -51792,7 +51907,7 @@
       <c r="L533" s="169"/>
       <c r="M533" s="168"/>
     </row>
-    <row r="534" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="534" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A534" s="168" t="s">
         <v>3129</v>
       </c>
@@ -51809,7 +51924,7 @@
       <c r="L534" s="169"/>
       <c r="M534" s="168"/>
     </row>
-    <row r="535" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="535" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A535" s="168" t="s">
         <v>3130</v>
       </c>
@@ -51826,7 +51941,7 @@
       <c r="L535" s="169"/>
       <c r="M535" s="168"/>
     </row>
-    <row r="536" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="536" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A536" s="168" t="s">
         <v>3131</v>
       </c>
@@ -51843,7 +51958,7 @@
       <c r="L536" s="169"/>
       <c r="M536" s="168"/>
     </row>
-    <row r="537" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="537" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A537" s="168" t="s">
         <v>3132</v>
       </c>
@@ -51859,6 +51974,286 @@
       <c r="K537" s="169"/>
       <c r="L537" s="169"/>
       <c r="M537" s="168"/>
+    </row>
+    <row r="538" spans="1:19">
+      <c r="N538" s="175"/>
+      <c r="O538" s="175"/>
+      <c r="P538" s="175"/>
+      <c r="Q538" s="175"/>
+      <c r="R538" s="175"/>
+      <c r="S538" s="175"/>
+    </row>
+    <row r="539" spans="1:19">
+      <c r="N539" s="175"/>
+      <c r="O539" s="175"/>
+      <c r="P539" s="175"/>
+      <c r="Q539" s="175"/>
+      <c r="R539" s="175"/>
+      <c r="S539" s="175"/>
+    </row>
+    <row r="540" spans="1:19">
+      <c r="N540" s="175"/>
+      <c r="O540" s="175"/>
+      <c r="P540" s="175"/>
+      <c r="Q540" s="175"/>
+      <c r="R540" s="175"/>
+      <c r="S540" s="175"/>
+    </row>
+    <row r="541" spans="1:19">
+      <c r="N541" s="175"/>
+      <c r="O541" s="175"/>
+      <c r="P541" s="175"/>
+      <c r="Q541" s="175"/>
+      <c r="R541" s="175"/>
+      <c r="S541" s="175"/>
+    </row>
+    <row r="542" spans="1:19">
+      <c r="N542" s="175"/>
+      <c r="O542" s="175"/>
+      <c r="P542" s="175"/>
+      <c r="Q542" s="175"/>
+      <c r="R542" s="175"/>
+      <c r="S542" s="175"/>
+    </row>
+    <row r="543" spans="1:19">
+      <c r="N543" s="175"/>
+      <c r="O543" s="175"/>
+      <c r="P543" s="175"/>
+      <c r="Q543" s="175"/>
+      <c r="R543" s="175"/>
+      <c r="S543" s="175"/>
+    </row>
+    <row r="544" spans="1:19">
+      <c r="N544" s="175"/>
+      <c r="O544" s="175"/>
+      <c r="P544" s="175"/>
+      <c r="Q544" s="175"/>
+      <c r="R544" s="175"/>
+      <c r="S544" s="175"/>
+    </row>
+    <row r="545" spans="14:19">
+      <c r="N545" s="175"/>
+      <c r="O545" s="175"/>
+      <c r="P545" s="175"/>
+      <c r="Q545" s="175"/>
+      <c r="R545" s="175"/>
+      <c r="S545" s="175"/>
+    </row>
+    <row r="546" spans="14:19">
+      <c r="N546" s="175"/>
+      <c r="O546" s="175"/>
+      <c r="P546" s="175"/>
+      <c r="Q546" s="175"/>
+      <c r="R546" s="175"/>
+      <c r="S546" s="175"/>
+    </row>
+    <row r="547" spans="14:19">
+      <c r="N547" s="175"/>
+      <c r="O547" s="175"/>
+      <c r="P547" s="175"/>
+      <c r="Q547" s="175"/>
+      <c r="R547" s="175"/>
+      <c r="S547" s="175"/>
+    </row>
+    <row r="548" spans="14:19">
+      <c r="N548" s="175"/>
+      <c r="O548" s="175"/>
+      <c r="P548" s="175"/>
+      <c r="Q548" s="175"/>
+      <c r="R548" s="175"/>
+      <c r="S548" s="175"/>
+    </row>
+    <row r="549" spans="14:19">
+      <c r="N549" s="175"/>
+      <c r="O549" s="175"/>
+      <c r="P549" s="175"/>
+      <c r="Q549" s="175"/>
+      <c r="R549" s="175"/>
+      <c r="S549" s="175"/>
+    </row>
+    <row r="550" spans="14:19">
+      <c r="N550" s="175"/>
+      <c r="O550" s="175"/>
+      <c r="P550" s="175"/>
+      <c r="Q550" s="175"/>
+      <c r="R550" s="175"/>
+      <c r="S550" s="175"/>
+    </row>
+    <row r="551" spans="14:19">
+      <c r="N551" s="175"/>
+      <c r="O551" s="175"/>
+      <c r="P551" s="175"/>
+      <c r="Q551" s="175"/>
+      <c r="R551" s="175"/>
+      <c r="S551" s="175"/>
+    </row>
+    <row r="552" spans="14:19">
+      <c r="N552" s="175"/>
+      <c r="O552" s="175"/>
+      <c r="P552" s="175"/>
+      <c r="Q552" s="175"/>
+      <c r="R552" s="175"/>
+      <c r="S552" s="175"/>
+    </row>
+    <row r="553" spans="14:19">
+      <c r="N553" s="175"/>
+      <c r="O553" s="175"/>
+      <c r="P553" s="175"/>
+      <c r="Q553" s="175"/>
+      <c r="R553" s="175"/>
+      <c r="S553" s="175"/>
+    </row>
+    <row r="554" spans="14:19">
+      <c r="N554" s="175"/>
+      <c r="O554" s="175"/>
+      <c r="P554" s="175"/>
+      <c r="Q554" s="175"/>
+      <c r="R554" s="175"/>
+      <c r="S554" s="175"/>
+    </row>
+    <row r="555" spans="14:19">
+      <c r="N555" s="175"/>
+      <c r="O555" s="175"/>
+      <c r="P555" s="175"/>
+      <c r="Q555" s="175"/>
+      <c r="R555" s="175"/>
+      <c r="S555" s="175"/>
+    </row>
+    <row r="556" spans="14:19">
+      <c r="N556" s="175"/>
+      <c r="O556" s="175"/>
+      <c r="P556" s="175"/>
+      <c r="Q556" s="175"/>
+      <c r="R556" s="175"/>
+      <c r="S556" s="175"/>
+    </row>
+    <row r="557" spans="14:19">
+      <c r="N557" s="175"/>
+      <c r="O557" s="175"/>
+      <c r="P557" s="175"/>
+      <c r="Q557" s="175"/>
+      <c r="R557" s="175"/>
+      <c r="S557" s="175"/>
+    </row>
+    <row r="558" spans="14:19">
+      <c r="N558" s="175"/>
+      <c r="O558" s="175"/>
+      <c r="P558" s="175"/>
+      <c r="Q558" s="175"/>
+      <c r="R558" s="175"/>
+      <c r="S558" s="175"/>
+    </row>
+    <row r="559" spans="14:19">
+      <c r="N559" s="175"/>
+      <c r="O559" s="175"/>
+      <c r="P559" s="175"/>
+      <c r="Q559" s="175"/>
+      <c r="R559" s="175"/>
+      <c r="S559" s="175"/>
+    </row>
+    <row r="560" spans="14:19">
+      <c r="N560" s="175"/>
+      <c r="O560" s="175"/>
+      <c r="P560" s="175"/>
+      <c r="Q560" s="175"/>
+      <c r="R560" s="175"/>
+      <c r="S560" s="175"/>
+    </row>
+    <row r="561" spans="14:19">
+      <c r="N561" s="175"/>
+      <c r="O561" s="175"/>
+      <c r="P561" s="175"/>
+      <c r="Q561" s="175"/>
+      <c r="R561" s="175"/>
+      <c r="S561" s="175"/>
+    </row>
+    <row r="562" spans="14:19">
+      <c r="N562" s="175"/>
+      <c r="O562" s="175"/>
+      <c r="P562" s="175"/>
+      <c r="Q562" s="175"/>
+      <c r="R562" s="175"/>
+      <c r="S562" s="175"/>
+    </row>
+    <row r="563" spans="14:19">
+      <c r="N563" s="175"/>
+      <c r="O563" s="175"/>
+      <c r="P563" s="175"/>
+      <c r="Q563" s="175"/>
+      <c r="R563" s="175"/>
+      <c r="S563" s="175"/>
+    </row>
+    <row r="564" spans="14:19">
+      <c r="N564" s="175"/>
+      <c r="O564" s="175"/>
+      <c r="P564" s="175"/>
+      <c r="Q564" s="175"/>
+      <c r="R564" s="175"/>
+      <c r="S564" s="175"/>
+    </row>
+    <row r="565" spans="14:19">
+      <c r="N565" s="175"/>
+      <c r="O565" s="175"/>
+      <c r="P565" s="175"/>
+      <c r="Q565" s="175"/>
+      <c r="R565" s="175"/>
+      <c r="S565" s="175"/>
+    </row>
+    <row r="566" spans="14:19">
+      <c r="N566" s="175"/>
+      <c r="O566" s="175"/>
+      <c r="P566" s="175"/>
+      <c r="Q566" s="175"/>
+      <c r="R566" s="175"/>
+      <c r="S566" s="175"/>
+    </row>
+    <row r="567" spans="14:19">
+      <c r="N567" s="175"/>
+      <c r="O567" s="175"/>
+      <c r="P567" s="175"/>
+      <c r="Q567" s="175"/>
+      <c r="R567" s="175"/>
+      <c r="S567" s="175"/>
+    </row>
+    <row r="568" spans="14:19">
+      <c r="N568" s="175"/>
+      <c r="O568" s="175"/>
+      <c r="P568" s="175"/>
+      <c r="Q568" s="175"/>
+      <c r="R568" s="175"/>
+      <c r="S568" s="175"/>
+    </row>
+    <row r="569" spans="14:19">
+      <c r="N569" s="175"/>
+      <c r="O569" s="175"/>
+      <c r="P569" s="175"/>
+      <c r="Q569" s="175"/>
+      <c r="R569" s="175"/>
+      <c r="S569" s="175"/>
+    </row>
+    <row r="570" spans="14:19">
+      <c r="N570" s="175"/>
+      <c r="O570" s="175"/>
+      <c r="P570" s="175"/>
+      <c r="Q570" s="175"/>
+      <c r="R570" s="175"/>
+      <c r="S570" s="175"/>
+    </row>
+    <row r="571" spans="14:19">
+      <c r="N571" s="175"/>
+      <c r="O571" s="175"/>
+      <c r="P571" s="175"/>
+      <c r="Q571" s="175"/>
+      <c r="R571" s="175"/>
+      <c r="S571" s="175"/>
+    </row>
+    <row r="572" spans="14:19">
+      <c r="N572" s="175"/>
+      <c r="O572" s="175"/>
+      <c r="P572" s="175"/>
+      <c r="Q572" s="175"/>
+      <c r="R572" s="175"/>
+      <c r="S572" s="175"/>
     </row>
     <row r="1044938" spans="2:3">
       <c r="C1044938" s="6"/>

</xml_diff>